<commit_message>
Feat : HP, MP 리젠 추가
</commit_message>
<xml_diff>
--- a/DesignData/Excel_Masters/ArmorStats_Master.xlsx
+++ b/DesignData/Excel_Masters/ArmorStats_Master.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="76">
   <si>
     <t>---</t>
   </si>
@@ -241,6 +241,12 @@
   </si>
   <si>
     <t>군대를 호령하던 위대한 지휘관의 권위가 담겨 있습니다.</t>
+  </si>
+  <si>
+    <t>HealthRegen</t>
+  </si>
+  <si>
+    <t>ManaRegen</t>
   </si>
 </sst>
 </file>
@@ -1158,10 +1164,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1175,22 +1181,28 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1203,23 +1215,29 @@
       <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
         <v>38</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>56</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>10</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>11</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1232,23 +1250,29 @@
       <c r="D3">
         <v>50</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
         <v>39</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>57</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>14</v>
       </c>
-      <c r="H3" t="s">
+      <c r="J3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1261,23 +1285,29 @@
       <c r="D4">
         <v>0</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
         <v>40</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>58</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>14</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>15</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1290,23 +1320,29 @@
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5" t="s">
         <v>41</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>59</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>14</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>15</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1319,23 +1355,29 @@
       <c r="D6">
         <v>150</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
         <v>42</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>60</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>20</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>15</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1348,23 +1390,29 @@
       <c r="D7">
         <v>50</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>61</v>
       </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>23</v>
       </c>
-      <c r="H7" t="s">
+      <c r="J7" t="s">
         <v>15</v>
       </c>
-      <c r="I7" t="s">
+      <c r="K7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1377,23 +1425,29 @@
       <c r="D8">
         <v>40</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
         <v>44</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>62</v>
       </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
         <v>14</v>
       </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>11</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -1406,23 +1460,29 @@
       <c r="D9">
         <v>20</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s">
         <v>45</v>
       </c>
-      <c r="F9" t="s">
+      <c r="H9" t="s">
         <v>63</v>
       </c>
-      <c r="G9" t="s">
+      <c r="I9" t="s">
         <v>27</v>
       </c>
-      <c r="H9" t="s">
+      <c r="J9" t="s">
         <v>15</v>
       </c>
-      <c r="I9" t="s">
+      <c r="K9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1435,23 +1495,29 @@
       <c r="D10">
         <v>60</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10" t="s">
         <v>46</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" t="s">
         <v>64</v>
       </c>
-      <c r="G10" t="s">
+      <c r="I10" t="s">
         <v>20</v>
       </c>
-      <c r="H10" t="s">
+      <c r="J10" t="s">
         <v>15</v>
       </c>
-      <c r="I10" t="s">
+      <c r="K10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1464,23 +1530,29 @@
       <c r="D11">
         <v>80</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11" t="s">
         <v>47</v>
       </c>
-      <c r="F11" t="s">
+      <c r="H11" t="s">
         <v>65</v>
       </c>
-      <c r="G11" t="s">
+      <c r="I11" t="s">
         <v>23</v>
       </c>
-      <c r="H11" t="s">
+      <c r="J11" t="s">
         <v>15</v>
       </c>
-      <c r="I11" t="s">
+      <c r="K11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -1493,23 +1565,29 @@
       <c r="D12">
         <v>50</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12" t="s">
         <v>48</v>
       </c>
-      <c r="F12" t="s">
+      <c r="H12" t="s">
         <v>66</v>
       </c>
-      <c r="G12" t="s">
+      <c r="I12" t="s">
         <v>27</v>
       </c>
-      <c r="H12" t="s">
+      <c r="J12" t="s">
         <v>11</v>
       </c>
-      <c r="I12" t="s">
+      <c r="K12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1522,23 +1600,29 @@
       <c r="D13">
         <v>0</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s">
         <v>49</v>
       </c>
-      <c r="F13" t="s">
+      <c r="H13" t="s">
         <v>67</v>
       </c>
-      <c r="G13" t="s">
+      <c r="I13" t="s">
         <v>14</v>
       </c>
-      <c r="H13" t="s">
+      <c r="J13" t="s">
         <v>15</v>
       </c>
-      <c r="I13" t="s">
+      <c r="K13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1551,23 +1635,29 @@
       <c r="D14">
         <v>150</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14" t="s">
         <v>50</v>
       </c>
-      <c r="F14" t="s">
+      <c r="H14" t="s">
         <v>68</v>
       </c>
-      <c r="G14" t="s">
+      <c r="I14" t="s">
         <v>20</v>
       </c>
-      <c r="H14" t="s">
+      <c r="J14" t="s">
         <v>15</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1580,23 +1670,29 @@
       <c r="D15">
         <v>120</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s">
         <v>51</v>
       </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>69</v>
       </c>
-      <c r="G15" t="s">
+      <c r="I15" t="s">
         <v>23</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" t="s">
         <v>15</v>
       </c>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -1609,23 +1705,29 @@
       <c r="D16">
         <v>20</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s">
         <v>52</v>
       </c>
-      <c r="F16" t="s">
+      <c r="H16" t="s">
         <v>70</v>
       </c>
-      <c r="G16" t="s">
+      <c r="I16" t="s">
         <v>14</v>
       </c>
-      <c r="H16" t="s">
+      <c r="J16" t="s">
         <v>11</v>
       </c>
-      <c r="I16" t="s">
+      <c r="K16" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -1638,23 +1740,29 @@
       <c r="D17">
         <v>0</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17" t="s">
         <v>53</v>
       </c>
-      <c r="F17" t="s">
+      <c r="H17" t="s">
         <v>71</v>
       </c>
-      <c r="G17" t="s">
+      <c r="I17" t="s">
         <v>14</v>
       </c>
-      <c r="H17" t="s">
+      <c r="J17" t="s">
         <v>15</v>
       </c>
-      <c r="I17" t="s">
+      <c r="K17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -1667,23 +1775,29 @@
       <c r="D18">
         <v>30</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" t="s">
         <v>54</v>
       </c>
-      <c r="F18" t="s">
+      <c r="H18" t="s">
         <v>72</v>
       </c>
-      <c r="G18" t="s">
+      <c r="I18" t="s">
         <v>20</v>
       </c>
-      <c r="H18" t="s">
+      <c r="J18" t="s">
         <v>15</v>
       </c>
-      <c r="I18" t="s">
+      <c r="K18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1696,19 +1810,25 @@
       <c r="D19">
         <v>80</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" t="s">
         <v>55</v>
       </c>
-      <c r="F19" t="s">
+      <c r="H19" t="s">
         <v>73</v>
       </c>
-      <c r="G19" t="s">
+      <c r="I19" t="s">
         <v>23</v>
       </c>
-      <c r="H19" t="s">
+      <c r="J19" t="s">
         <v>15</v>
       </c>
-      <c r="I19" t="s">
+      <c r="K19" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>